<commit_message>
French: Edit long text into short form
</commit_message>
<xml_diff>
--- a/Trans To Vostok/French/Glossary.xlsx
+++ b/Trans To Vostok/French/Glossary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SteamLibrary\steamapps\common\Road to Vostok\mods\Trans To Vostok\Trans To Vostok\French\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F793F567-EDCE-4D31-B610-8B4ED09EEF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6F61D7-3FFD-48EA-82C6-B4290ACE1C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -131,27 +131,18 @@
     <t>Highway</t>
   </si>
   <si>
-    <t>Autoroute</t>
-  </si>
-  <si>
     <t>mid-zone; connects Village/School</t>
   </si>
   <si>
     <t>School</t>
   </si>
   <si>
-    <t>École</t>
-  </si>
-  <si>
     <t>mid-zone; trader Doctor returns here</t>
   </si>
   <si>
     <t>Border Zone</t>
   </si>
   <si>
-    <t>Zone frontalière</t>
-  </si>
-  <si>
     <t>same as above</t>
   </si>
   <si>
@@ -167,9 +158,6 @@
     <t>Minefield</t>
   </si>
   <si>
-    <t>Champ de mines</t>
-  </si>
-  <si>
     <t>dangerous zone east of Outpost</t>
   </si>
   <si>
@@ -458,30 +446,15 @@
     <t>Vital of stamina (Hunger)</t>
   </si>
   <si>
-    <t>Hydration</t>
-  </si>
-  <si>
-    <t>Hydratation</t>
-  </si>
-  <si>
     <t>Vital of Thirst</t>
   </si>
   <si>
-    <t>Mental</t>
-  </si>
-  <si>
-    <t>Psychologique</t>
-  </si>
-  <si>
     <t>Vital of Mental health</t>
   </si>
   <si>
     <t>Body Temp</t>
   </si>
   <si>
-    <t>Température corporelle</t>
-  </si>
-  <si>
     <t>Vital of Body Temperature</t>
   </si>
   <si>
@@ -564,12 +537,6 @@
   </si>
   <si>
     <t>Statistiques de progression</t>
-  </si>
-  <si>
-    <t>Shelters</t>
-  </si>
-  <si>
-    <t>Refuges</t>
   </si>
   <si>
     <t xml:space="preserve">This is the number of unlocked "Shelters". Since this is the plural form of "Shelter", please be careful not to confuse it with other words. </t>
@@ -1025,6 +992,50 @@
   </si>
   <si>
     <t>Vision Nocturne</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Autoroute</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>École</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Village</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zone frontalière</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Champ de mines</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hydration</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Refuges</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shelters</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Temp.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Eau</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mental</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1466,7 +1477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1601,6 +1612,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1992,16 +2006,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="13" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2009,13 +2023,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2023,13 +2037,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="C3" s="18">
         <v>46135</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2037,13 +2051,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C4" s="18">
         <v>46147</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2051,13 +2065,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="C5" s="19">
         <v>2.7083333333333331E-2</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2065,13 +2079,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="38.4" customHeight="1">
@@ -2079,10 +2093,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="38.4" customHeight="1">
@@ -2090,13 +2104,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -2186,7 +2200,7 @@
       <c r="I2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="46" t="s">
         <v>14</v>
       </c>
       <c r="K2" s="8" t="s">
@@ -2221,7 +2235,7 @@
       <c r="I3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="46" t="s">
         <v>18</v>
       </c>
       <c r="K3" s="8" t="e">
@@ -2256,7 +2270,7 @@
       <c r="I4" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="46" t="s">
         <v>21</v>
       </c>
       <c r="K4" s="8" t="s">
@@ -2291,7 +2305,7 @@
       <c r="I5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="46" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2323,7 +2337,7 @@
       <c r="I6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="46" t="s">
         <v>28</v>
       </c>
     </row>
@@ -2355,7 +2369,7 @@
       <c r="I7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="46" t="s">
         <v>30</v>
       </c>
       <c r="K7" s="8" t="s">
@@ -2390,8 +2404,8 @@
       <c r="I8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="J8" t="s">
-        <v>33</v>
+      <c r="J8" s="46" t="s">
+        <v>325</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>34</v>
@@ -2425,11 +2439,11 @@
       <c r="I9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="46" t="s">
+        <v>323</v>
+      </c>
+      <c r="K9" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2458,13 +2472,13 @@
         <v>29</v>
       </c>
       <c r="I10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="J10" s="46" t="s">
+        <v>324</v>
+      </c>
+      <c r="K10" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="J10" t="s">
-        <v>39</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2490,16 +2504,16 @@
         <v>24</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="J11" t="s">
-        <v>42</v>
+        <v>39</v>
+      </c>
+      <c r="J11" s="46" t="s">
+        <v>326</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2525,16 +2539,16 @@
         <v>32</v>
       </c>
       <c r="H12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I12" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="I12" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="J12" t="s">
-        <v>45</v>
+      <c r="J12" s="46" t="s">
+        <v>42</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2560,16 +2574,16 @@
         <v>32</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="J13" t="s">
-        <v>48</v>
+        <v>44</v>
+      </c>
+      <c r="J13" s="46" t="s">
+        <v>327</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2595,16 +2609,16 @@
         <v>24</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="J14" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="J14" s="46" t="s">
+        <v>46</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2630,16 +2644,16 @@
         <v>32</v>
       </c>
       <c r="H15" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="46" t="s">
+        <v>49</v>
+      </c>
+      <c r="K15" s="8" t="s">
         <v>50</v>
-      </c>
-      <c r="I15" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="J15" t="s">
-        <v>53</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2665,16 +2679,16 @@
         <v>32</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="J16" t="s">
-        <v>55</v>
+        <v>51</v>
+      </c>
+      <c r="J16" s="46" t="s">
+        <v>51</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2697,19 +2711,19 @@
         <v>23</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="J17" t="s">
-        <v>58</v>
+        <v>53</v>
+      </c>
+      <c r="J17" s="46" t="s">
+        <v>54</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2732,19 +2746,19 @@
         <v>23</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H18" s="6" t="s">
         <v>29</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="J18" t="s">
-        <v>61</v>
+        <v>56</v>
+      </c>
+      <c r="J18" s="46" t="s">
+        <v>57</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2767,19 +2781,19 @@
         <v>23</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>29</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="J19" t="s">
-        <v>64</v>
+        <v>59</v>
+      </c>
+      <c r="J19" s="46" t="s">
+        <v>60</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2802,19 +2816,19 @@
         <v>23</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>29</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="J20" t="s">
-        <v>67</v>
+        <v>62</v>
+      </c>
+      <c r="J20" s="46" t="s">
+        <v>63</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2837,19 +2851,19 @@
         <v>23</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="J21" t="s">
-        <v>70</v>
+        <v>65</v>
+      </c>
+      <c r="J21" s="46" t="s">
+        <v>66</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2872,19 +2886,19 @@
         <v>23</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="J22" t="s">
-        <v>72</v>
+        <v>68</v>
+      </c>
+      <c r="J22" s="46" t="s">
+        <v>68</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2907,19 +2921,19 @@
         <v>23</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="J23" t="s">
-        <v>75</v>
+        <v>70</v>
+      </c>
+      <c r="J23" s="46" t="s">
+        <v>71</v>
       </c>
       <c r="K23" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2942,16 +2956,16 @@
         <v>23</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="J24" t="s">
-        <v>75</v>
+        <v>70</v>
+      </c>
+      <c r="J24" s="46" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -2974,19 +2988,19 @@
         <v>23</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H25" s="40" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I25" s="42" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="J25" s="43" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K25" s="44" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -3006,22 +3020,22 @@
         <v>0</v>
       </c>
       <c r="F26" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="G26" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="H26" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="I26" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="J26" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="K26" s="36" t="s">
         <v>80</v>
-      </c>
-      <c r="G26" s="31" t="s">
-        <v>81</v>
-      </c>
-      <c r="H26" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="I26" s="34" t="s">
-        <v>82</v>
-      </c>
-      <c r="J26" s="35" t="s">
-        <v>83</v>
-      </c>
-      <c r="K26" s="36" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -3041,22 +3055,22 @@
         <v>0</v>
       </c>
       <c r="F27" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="J27" t="s">
-        <v>85</v>
+        <v>81</v>
+      </c>
+      <c r="J27" s="46" t="s">
+        <v>81</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -3076,22 +3090,22 @@
         <v>0</v>
       </c>
       <c r="F28" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>29</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="J28" t="s">
-        <v>89</v>
+        <v>84</v>
+      </c>
+      <c r="J28" s="46" t="s">
+        <v>85</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -3111,22 +3125,22 @@
         <v>0</v>
       </c>
       <c r="F29" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H29" s="6" t="s">
         <v>29</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="J29" t="s">
-        <v>92</v>
+        <v>87</v>
+      </c>
+      <c r="J29" s="46" t="s">
+        <v>88</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -3146,22 +3160,22 @@
         <v>0</v>
       </c>
       <c r="F30" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="J30" t="s">
-        <v>95</v>
+        <v>90</v>
+      </c>
+      <c r="J30" s="46" t="s">
+        <v>91</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -3181,22 +3195,22 @@
         <v>0</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I31" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="J31" t="s">
-        <v>98</v>
+        <v>93</v>
+      </c>
+      <c r="J31" s="46" t="s">
+        <v>94</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -3216,22 +3230,22 @@
         <v>0</v>
       </c>
       <c r="F32" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="J32" t="s">
-        <v>101</v>
+        <v>96</v>
+      </c>
+      <c r="J32" s="46" t="s">
+        <v>97</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -3251,22 +3265,22 @@
         <v>0</v>
       </c>
       <c r="F33" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H33" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="J33" t="s">
-        <v>104</v>
+        <v>99</v>
+      </c>
+      <c r="J33" s="46" t="s">
+        <v>100</v>
       </c>
       <c r="K33" s="8" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -3286,22 +3300,22 @@
         <v>0</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="J34" t="s">
-        <v>107</v>
+        <v>102</v>
+      </c>
+      <c r="J34" s="46" t="s">
+        <v>103</v>
       </c>
       <c r="K34" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -3321,22 +3335,22 @@
         <v>0</v>
       </c>
       <c r="F35" s="41" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H35" s="40" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I35" s="42" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="J35" s="43" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="K35" s="44" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -3356,22 +3370,22 @@
         <v>0</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>29</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="J36" t="s">
-        <v>114</v>
+        <v>110</v>
+      </c>
+      <c r="J36" s="46" t="s">
+        <v>110</v>
       </c>
       <c r="K36" s="8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -3391,22 +3405,22 @@
         <v>0</v>
       </c>
       <c r="F37" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I37" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="J37" s="46" t="s">
         <v>113</v>
       </c>
-      <c r="H37" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="I37" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="J37" t="s">
-        <v>117</v>
-      </c>
       <c r="K37" s="8" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -3426,22 +3440,22 @@
         <v>0</v>
       </c>
       <c r="F38" s="26" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="J38" t="s">
-        <v>120</v>
+        <v>115</v>
+      </c>
+      <c r="J38" s="46" t="s">
+        <v>116</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -3461,10 +3475,10 @@
         <v>0</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="J39" t="s">
-        <v>120</v>
+        <v>115</v>
+      </c>
+      <c r="J39" s="46" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="40" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -3484,22 +3498,22 @@
         <v>0</v>
       </c>
       <c r="F40" s="41" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G40" s="39" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H40" s="40" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="I40" s="42" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J40" s="43" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="K40" s="44" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -3519,22 +3533,22 @@
         <v>0</v>
       </c>
       <c r="F41" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="G41" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="H41" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="I41" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="J41" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="G41" s="31" t="s">
+      <c r="K41" s="36" t="s">
         <v>127</v>
-      </c>
-      <c r="H41" s="32" t="s">
-        <v>128</v>
-      </c>
-      <c r="I41" s="34" t="s">
-        <v>129</v>
-      </c>
-      <c r="J41" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="K41" s="36" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -3554,22 +3568,22 @@
         <v>0</v>
       </c>
       <c r="F42" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="J42" t="s">
-        <v>134</v>
+        <v>128</v>
+      </c>
+      <c r="J42" s="46" t="s">
+        <v>130</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -3589,22 +3603,22 @@
         <v>0</v>
       </c>
       <c r="F43" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G43" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H43" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="H43" s="6" t="s">
-        <v>136</v>
-      </c>
       <c r="I43" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="J43" t="s">
-        <v>138</v>
+        <v>133</v>
+      </c>
+      <c r="J43" s="46" t="s">
+        <v>134</v>
       </c>
       <c r="K43" s="8" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -3624,22 +3638,22 @@
         <v>0</v>
       </c>
       <c r="F44" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="J44" t="s">
-        <v>140</v>
+        <v>135</v>
+      </c>
+      <c r="J44" s="46" t="s">
+        <v>136</v>
       </c>
       <c r="K44" s="8" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -3659,22 +3673,22 @@
         <v>0</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I45" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="J45" t="s">
-        <v>143</v>
+        <v>138</v>
+      </c>
+      <c r="J45" s="46" t="s">
+        <v>139</v>
       </c>
       <c r="K45" s="8" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3685,7 +3699,7 @@
         <v>0</v>
       </c>
       <c r="C46" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" s="1">
         <v>0</v>
@@ -3694,22 +3708,22 @@
         <v>0</v>
       </c>
       <c r="F46" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="J46" t="s">
-        <v>146</v>
+        <v>328</v>
+      </c>
+      <c r="J46" s="46" t="s">
+        <v>332</v>
       </c>
       <c r="K46" s="8" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -3720,7 +3734,7 @@
         <v>0</v>
       </c>
       <c r="C47" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47" s="1">
         <v>0</v>
@@ -3729,22 +3743,22 @@
         <v>0</v>
       </c>
       <c r="F47" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J47" t="s">
-        <v>149</v>
+        <v>333</v>
+      </c>
+      <c r="J47" s="46" t="s">
+        <v>333</v>
       </c>
       <c r="K47" s="8" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3755,7 +3769,7 @@
         <v>0</v>
       </c>
       <c r="C48" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" s="1">
         <v>0</v>
@@ -3764,22 +3778,22 @@
         <v>0</v>
       </c>
       <c r="F48" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="J48" t="s">
-        <v>152</v>
+        <v>143</v>
+      </c>
+      <c r="J48" s="46" t="s">
+        <v>331</v>
       </c>
       <c r="K48" s="8" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3799,22 +3813,22 @@
         <v>0</v>
       </c>
       <c r="F49" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I49" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="J49" t="s">
-        <v>83</v>
+        <v>78</v>
+      </c>
+      <c r="J49" s="46" t="s">
+        <v>79</v>
       </c>
       <c r="K49" s="8" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3834,19 +3848,19 @@
         <v>0</v>
       </c>
       <c r="F50" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="J50" t="s">
-        <v>157</v>
+        <v>147</v>
+      </c>
+      <c r="J50" s="46" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3866,19 +3880,19 @@
         <v>0</v>
       </c>
       <c r="F51" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="J51" t="s">
-        <v>159</v>
+        <v>149</v>
+      </c>
+      <c r="J51" s="46" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3898,19 +3912,19 @@
         <v>0</v>
       </c>
       <c r="F52" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="J52" t="s">
-        <v>161</v>
+        <v>151</v>
+      </c>
+      <c r="J52" s="46" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3930,19 +3944,19 @@
         <v>0</v>
       </c>
       <c r="F53" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I53" s="10" t="s">
-        <v>162</v>
-      </c>
-      <c r="J53" t="s">
-        <v>163</v>
+        <v>153</v>
+      </c>
+      <c r="J53" s="46" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -3962,19 +3976,19 @@
         <v>0</v>
       </c>
       <c r="F54" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G54" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="I54" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="H54" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="I54" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="J54" t="s">
-        <v>165</v>
+      <c r="J54" s="46" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -3994,19 +4008,19 @@
         <v>0</v>
       </c>
       <c r="F55" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I55" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="J55" t="s">
-        <v>166</v>
+        <v>157</v>
+      </c>
+      <c r="J55" s="46" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -4026,19 +4040,19 @@
         <v>0</v>
       </c>
       <c r="F56" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>167</v>
-      </c>
-      <c r="J56" t="s">
-        <v>168</v>
+        <v>158</v>
+      </c>
+      <c r="J56" s="46" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -4058,19 +4072,19 @@
         <v>0</v>
       </c>
       <c r="F57" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="J57" t="s">
-        <v>170</v>
+        <v>160</v>
+      </c>
+      <c r="J57" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -4090,19 +4104,19 @@
         <v>0</v>
       </c>
       <c r="F58" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="J58" t="s">
-        <v>172</v>
+        <v>162</v>
+      </c>
+      <c r="J58" s="46" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -4122,19 +4136,19 @@
         <v>0</v>
       </c>
       <c r="F59" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="J59" t="s">
-        <v>174</v>
+        <v>164</v>
+      </c>
+      <c r="J59" s="46" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -4154,19 +4168,19 @@
         <v>0</v>
       </c>
       <c r="F60" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="J60" t="s">
-        <v>175</v>
+        <v>166</v>
+      </c>
+      <c r="J60" s="46" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -4186,19 +4200,19 @@
         <v>0</v>
       </c>
       <c r="F61" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I61" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="J61" t="s">
-        <v>177</v>
+        <v>167</v>
+      </c>
+      <c r="J61" s="46" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -4218,19 +4232,19 @@
         <v>0</v>
       </c>
       <c r="F62" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="J62" t="s">
-        <v>180</v>
+        <v>170</v>
+      </c>
+      <c r="J62" s="46" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="38.4" customHeight="1">
@@ -4250,22 +4264,22 @@
         <v>0</v>
       </c>
       <c r="F63" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="J63" t="s">
-        <v>182</v>
+        <v>330</v>
+      </c>
+      <c r="J63" s="46" t="s">
+        <v>329</v>
       </c>
       <c r="K63" s="8" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -4285,19 +4299,19 @@
         <v>0</v>
       </c>
       <c r="F64" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="J64" t="s">
-        <v>185</v>
+        <v>173</v>
+      </c>
+      <c r="J64" s="46" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -4317,19 +4331,19 @@
         <v>0</v>
       </c>
       <c r="F65" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I65" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="J65" t="s">
-        <v>187</v>
+        <v>175</v>
+      </c>
+      <c r="J65" s="46" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="38.4" customHeight="1">
@@ -4349,22 +4363,22 @@
         <v>0</v>
       </c>
       <c r="F66" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G66" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I66" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="J66" s="46" t="s">
         <v>178</v>
       </c>
-      <c r="H66" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="I66" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="J66" t="s">
-        <v>189</v>
-      </c>
       <c r="K66" s="8" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
     </row>
     <row r="67" spans="1:11">
@@ -4384,22 +4398,22 @@
         <v>0</v>
       </c>
       <c r="F67" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="I67" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="J67" t="s">
-        <v>192</v>
+        <v>180</v>
+      </c>
+      <c r="J67" s="46" t="s">
+        <v>181</v>
       </c>
       <c r="K67" s="8" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -4419,19 +4433,19 @@
         <v>0</v>
       </c>
       <c r="F68" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="J68" t="s">
-        <v>196</v>
+        <v>184</v>
+      </c>
+      <c r="J68" s="46" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -4451,19 +4465,19 @@
         <v>0</v>
       </c>
       <c r="F69" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="I69" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="J69" t="s">
-        <v>198</v>
+        <v>186</v>
+      </c>
+      <c r="J69" s="46" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -4483,19 +4497,19 @@
         <v>0</v>
       </c>
       <c r="F70" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="J70" t="s">
-        <v>200</v>
+        <v>188</v>
+      </c>
+      <c r="J70" s="46" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -4515,19 +4529,19 @@
         <v>0</v>
       </c>
       <c r="F71" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="I71" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="J71" t="s">
-        <v>202</v>
+        <v>190</v>
+      </c>
+      <c r="J71" s="46" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -4547,19 +4561,19 @@
         <v>0</v>
       </c>
       <c r="F72" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="J72" t="s">
-        <v>205</v>
+        <v>193</v>
+      </c>
+      <c r="J72" s="46" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -4579,19 +4593,19 @@
         <v>0</v>
       </c>
       <c r="F73" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="J73" t="s">
-        <v>207</v>
+        <v>195</v>
+      </c>
+      <c r="J73" s="46" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -4611,19 +4625,19 @@
         <v>0</v>
       </c>
       <c r="F74" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="J74" t="s">
-        <v>209</v>
+        <v>197</v>
+      </c>
+      <c r="J74" s="46" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -4643,19 +4657,19 @@
         <v>0</v>
       </c>
       <c r="F75" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I75" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="J75" t="s">
-        <v>212</v>
+        <v>200</v>
+      </c>
+      <c r="J75" s="46" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -4675,19 +4689,19 @@
         <v>0</v>
       </c>
       <c r="F76" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="J76" t="s">
-        <v>215</v>
+        <v>203</v>
+      </c>
+      <c r="J76" s="46" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="77" spans="1:11">
@@ -4707,22 +4721,22 @@
         <v>0</v>
       </c>
       <c r="F77" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="J77" t="s">
-        <v>217</v>
+        <v>205</v>
+      </c>
+      <c r="J77" s="46" t="s">
+        <v>206</v>
       </c>
       <c r="K77" s="8" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -4742,19 +4756,19 @@
         <v>0</v>
       </c>
       <c r="F78" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="J78" t="s">
-        <v>220</v>
+        <v>208</v>
+      </c>
+      <c r="J78" s="46" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="79" spans="1:11">
@@ -4774,19 +4788,19 @@
         <v>0</v>
       </c>
       <c r="F79" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G79" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="I79" s="10" t="s">
         <v>210</v>
       </c>
-      <c r="H79" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="I79" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="J79" t="s">
-        <v>221</v>
+      <c r="J79" s="46" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="80" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -4806,22 +4820,22 @@
         <v>0</v>
       </c>
       <c r="F80" s="41" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G80" s="39" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="H80" s="40" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="I80" s="42" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="J80" s="43" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="K80" s="44" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
     </row>
     <row r="81" spans="1:11">
@@ -4841,22 +4855,22 @@
         <v>0</v>
       </c>
       <c r="F81" s="33" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G81" s="31" t="s">
+        <v>202</v>
+      </c>
+      <c r="H81" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="H81" s="32" t="s">
-        <v>224</v>
-      </c>
       <c r="I81" s="34" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="J81" s="35" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="K81" s="36" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -4876,22 +4890,22 @@
         <v>0</v>
       </c>
       <c r="F82" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G82" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H82" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I82" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="J82" t="s">
-        <v>229</v>
+        <v>217</v>
+      </c>
+      <c r="J82" s="46" t="s">
+        <v>218</v>
       </c>
       <c r="K82" s="8" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
     </row>
     <row r="83" spans="1:11">
@@ -4911,22 +4925,22 @@
         <v>0</v>
       </c>
       <c r="F83" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G83" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H83" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H83" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I83" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="J83" t="s">
-        <v>232</v>
+        <v>220</v>
+      </c>
+      <c r="J83" s="46" t="s">
+        <v>221</v>
       </c>
       <c r="K83" s="8" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" spans="1:11">
@@ -4946,22 +4960,22 @@
         <v>0</v>
       </c>
       <c r="F84" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G84" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H84" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H84" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I84" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="J84" t="s">
-        <v>234</v>
+        <v>223</v>
+      </c>
+      <c r="J84" s="46" t="s">
+        <v>223</v>
       </c>
       <c r="K84" s="8" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
     </row>
     <row r="85" spans="1:11">
@@ -4981,22 +4995,22 @@
         <v>0</v>
       </c>
       <c r="F85" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G85" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H85" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H85" s="6" t="s">
+      <c r="I85" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="J85" s="46" t="s">
+        <v>223</v>
+      </c>
+      <c r="K85" s="8" t="s">
         <v>224</v>
-      </c>
-      <c r="I85" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="J85" t="s">
-        <v>234</v>
-      </c>
-      <c r="K85" s="8" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -5016,22 +5030,22 @@
         <v>0</v>
       </c>
       <c r="F86" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G86" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H86" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H86" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I86" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="J86" t="s">
-        <v>234</v>
+        <v>223</v>
+      </c>
+      <c r="J86" s="46" t="s">
+        <v>223</v>
       </c>
       <c r="K86" s="8" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
     </row>
     <row r="87" spans="1:11">
@@ -5051,22 +5065,22 @@
         <v>0</v>
       </c>
       <c r="F87" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G87" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H87" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H87" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I87" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="J87" t="s">
-        <v>238</v>
+        <v>226</v>
+      </c>
+      <c r="J87" s="46" t="s">
+        <v>227</v>
       </c>
       <c r="K87" s="8" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
     </row>
     <row r="88" spans="1:11">
@@ -5086,22 +5100,22 @@
         <v>0</v>
       </c>
       <c r="F88" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G88" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H88" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H88" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I88" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="J88" t="s">
-        <v>241</v>
+        <v>229</v>
+      </c>
+      <c r="J88" s="46" t="s">
+        <v>230</v>
       </c>
       <c r="K88" s="8" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
     </row>
     <row r="89" spans="1:11">
@@ -5121,22 +5135,22 @@
         <v>0</v>
       </c>
       <c r="F89" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G89" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H89" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H89" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I89" s="10" t="s">
-        <v>243</v>
-      </c>
-      <c r="J89" t="s">
-        <v>244</v>
+        <v>232</v>
+      </c>
+      <c r="J89" s="46" t="s">
+        <v>233</v>
       </c>
       <c r="K89" s="8" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
     </row>
     <row r="90" spans="1:11">
@@ -5156,22 +5170,22 @@
         <v>0</v>
       </c>
       <c r="F90" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G90" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H90" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H90" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I90" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="J90" t="s">
-        <v>247</v>
+        <v>235</v>
+      </c>
+      <c r="J90" s="46" t="s">
+        <v>236</v>
       </c>
       <c r="K90" s="8" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -5191,22 +5205,22 @@
         <v>0</v>
       </c>
       <c r="F91" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G91" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H91" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H91" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I91" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="J91" t="s">
-        <v>250</v>
+        <v>238</v>
+      </c>
+      <c r="J91" s="46" t="s">
+        <v>239</v>
       </c>
       <c r="K91" s="8" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -5226,22 +5240,22 @@
         <v>0</v>
       </c>
       <c r="F92" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G92" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H92" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H92" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I92" s="10" t="s">
-        <v>252</v>
-      </c>
-      <c r="J92" t="s">
-        <v>253</v>
+        <v>241</v>
+      </c>
+      <c r="J92" s="46" t="s">
+        <v>242</v>
       </c>
       <c r="K92" s="8" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="93" spans="1:11">
@@ -5261,22 +5275,22 @@
         <v>0</v>
       </c>
       <c r="F93" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G93" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H93" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H93" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I93" s="10" t="s">
-        <v>255</v>
-      </c>
-      <c r="J93" t="s">
-        <v>256</v>
+        <v>244</v>
+      </c>
+      <c r="J93" s="46" t="s">
+        <v>245</v>
       </c>
       <c r="K93" s="8" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
     </row>
     <row r="94" spans="1:11">
@@ -5296,22 +5310,22 @@
         <v>0</v>
       </c>
       <c r="F94" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G94" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H94" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H94" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I94" s="10" t="s">
-        <v>258</v>
-      </c>
-      <c r="J94" t="s">
-        <v>259</v>
+        <v>247</v>
+      </c>
+      <c r="J94" s="46" t="s">
+        <v>248</v>
       </c>
       <c r="K94" s="8" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
     </row>
     <row r="95" spans="1:11">
@@ -5331,22 +5345,22 @@
         <v>0</v>
       </c>
       <c r="F95" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G95" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H95" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H95" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I95" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="J95" t="s">
-        <v>262</v>
+        <v>250</v>
+      </c>
+      <c r="J95" s="46" t="s">
+        <v>251</v>
       </c>
       <c r="K95" s="8" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
     </row>
     <row r="96" spans="1:11">
@@ -5366,22 +5380,22 @@
         <v>0</v>
       </c>
       <c r="F96" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G96" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H96" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H96" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I96" s="10" t="s">
-        <v>264</v>
-      </c>
-      <c r="J96" t="s">
-        <v>265</v>
+        <v>253</v>
+      </c>
+      <c r="J96" s="46" t="s">
+        <v>254</v>
       </c>
       <c r="K96" s="8" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
     </row>
     <row r="97" spans="1:11">
@@ -5401,22 +5415,22 @@
         <v>0</v>
       </c>
       <c r="F97" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G97" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H97" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H97" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I97" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="J97" t="s">
-        <v>268</v>
+        <v>256</v>
+      </c>
+      <c r="J97" s="46" t="s">
+        <v>257</v>
       </c>
       <c r="K97" s="8" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
     </row>
     <row r="98" spans="1:11">
@@ -5436,22 +5450,22 @@
         <v>0</v>
       </c>
       <c r="F98" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G98" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H98" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H98" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I98" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="J98" t="s">
-        <v>270</v>
+        <v>259</v>
+      </c>
+      <c r="J98" s="46" t="s">
+        <v>259</v>
       </c>
       <c r="K98" s="8" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
     </row>
     <row r="99" spans="1:11">
@@ -5471,22 +5485,22 @@
         <v>0</v>
       </c>
       <c r="F99" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G99" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H99" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H99" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I99" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="J99" t="s">
-        <v>333</v>
+        <v>259</v>
+      </c>
+      <c r="J99" s="46" t="s">
+        <v>322</v>
       </c>
       <c r="K99" s="8" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
     </row>
     <row r="100" spans="1:11">
@@ -5506,22 +5520,22 @@
         <v>0</v>
       </c>
       <c r="F100" s="26" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G100" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H100" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="H100" s="6" t="s">
-        <v>224</v>
-      </c>
       <c r="I100" s="10" t="s">
-        <v>273</v>
-      </c>
-      <c r="J100" t="s">
-        <v>274</v>
+        <v>262</v>
+      </c>
+      <c r="J100" s="46" t="s">
+        <v>263</v>
       </c>
       <c r="K100" s="8" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
     </row>
     <row r="101" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -5541,22 +5555,22 @@
         <v>0</v>
       </c>
       <c r="F101" s="41" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="G101" s="39" t="s">
+        <v>202</v>
+      </c>
+      <c r="H101" s="40" t="s">
         <v>213</v>
       </c>
-      <c r="H101" s="40" t="s">
-        <v>224</v>
-      </c>
       <c r="I101" s="42" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="J101" s="43" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="K101" s="44" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
     </row>
     <row r="102" spans="1:11">
@@ -5576,22 +5590,22 @@
         <v>0</v>
       </c>
       <c r="F102" s="26" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="G102" s="1" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="I102" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="J102" t="s">
-        <v>282</v>
+        <v>270</v>
+      </c>
+      <c r="J102" s="46" t="s">
+        <v>271</v>
       </c>
       <c r="K102" s="8" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
     </row>
     <row r="103" spans="1:11">
@@ -5611,22 +5625,22 @@
         <v>0</v>
       </c>
       <c r="F103" s="26" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="G103" s="1" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="H103" s="6" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="I103" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="J103" t="s">
-        <v>286</v>
+        <v>274</v>
+      </c>
+      <c r="J103" s="46" t="s">
+        <v>275</v>
       </c>
       <c r="K103" s="8" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
     </row>
     <row r="104" spans="1:11">
@@ -5646,19 +5660,19 @@
         <v>0</v>
       </c>
       <c r="F104" s="26" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="G104" s="1" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I104" s="10" t="s">
-        <v>291</v>
-      </c>
-      <c r="J104" t="s">
-        <v>292</v>
+        <v>280</v>
+      </c>
+      <c r="J104" s="46" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -5678,19 +5692,19 @@
         <v>0</v>
       </c>
       <c r="F105" s="26" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="G105" s="1" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="H105" s="6" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I105" s="10" t="s">
-        <v>293</v>
-      </c>
-      <c r="J105" t="s">
-        <v>294</v>
+        <v>282</v>
+      </c>
+      <c r="J105" s="46" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -5710,19 +5724,19 @@
         <v>0</v>
       </c>
       <c r="F106" s="26" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="G106" s="1" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I106" s="10" t="s">
-        <v>295</v>
-      </c>
-      <c r="J106" t="s">
-        <v>296</v>
+        <v>284</v>
+      </c>
+      <c r="J106" s="46" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -5742,19 +5756,19 @@
         <v>0</v>
       </c>
       <c r="F107" s="26" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="G107" s="1" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="H107" s="6" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I107" s="10" t="s">
-        <v>297</v>
-      </c>
-      <c r="J107" t="s">
-        <v>298</v>
+        <v>286</v>
+      </c>
+      <c r="J107" s="46" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -5774,19 +5788,19 @@
         <v>0</v>
       </c>
       <c r="F108" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="G108" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="G108" s="1" t="s">
-        <v>299</v>
-      </c>
       <c r="H108" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="I108" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="J108" s="46" t="s">
         <v>290</v>
-      </c>
-      <c r="I108" s="10" t="s">
-        <v>300</v>
-      </c>
-      <c r="J108" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -5806,19 +5820,19 @@
         <v>0</v>
       </c>
       <c r="F109" s="26" t="s">
+        <v>277</v>
+      </c>
+      <c r="G109" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="G109" s="1" t="s">
-        <v>299</v>
-      </c>
       <c r="H109" s="6" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I109" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="J109" t="s">
-        <v>303</v>
+        <v>291</v>
+      </c>
+      <c r="J109" s="46" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -5838,19 +5852,19 @@
         <v>0</v>
       </c>
       <c r="F110" s="26" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="G110" s="1" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="I110" s="10" t="s">
-        <v>304</v>
-      </c>
-      <c r="J110" t="s">
-        <v>305</v>
+        <v>293</v>
+      </c>
+      <c r="J110" s="46" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="111" spans="1:11">
@@ -5870,19 +5884,19 @@
         <v>0</v>
       </c>
       <c r="F111" s="26" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="G111" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H111" s="6" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="I111" s="10" t="s">
-        <v>308</v>
-      </c>
-      <c r="J111" t="s">
-        <v>309</v>
+        <v>297</v>
+      </c>
+      <c r="J111" s="46" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="112" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -5902,19 +5916,19 @@
         <v>0</v>
       </c>
       <c r="F112" s="41" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="G112" s="39" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="H112" s="40" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="I112" s="42" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="J112" s="43" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="K112" s="44"/>
     </row>

</xml_diff>

<commit_message>
0.4.5d: Add some missing strings to translate
</commit_message>
<xml_diff>
--- a/Trans To Vostok/French/Glossary.xlsx
+++ b/Trans To Vostok/French/Glossary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SteamLibrary\steamapps\common\Road to Vostok\mods\Trans To Vostok\Trans To Vostok\French\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6F61D7-3FFD-48EA-82C6-B4290ACE1C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92F8F2B1-7BEE-41E8-8C16-70C99F3463B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MetaData" sheetId="1" r:id="rId1"/>
@@ -836,9 +836,6 @@
     <t>Corpse</t>
   </si>
   <si>
-    <t>Cadavre</t>
-  </si>
-  <si>
     <t>Lootable Container</t>
   </si>
   <si>
@@ -1036,6 +1033,10 @@
   </si>
   <si>
     <t>Mental</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cadavre</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2006,16 +2007,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="D1" s="13" t="s">
         <v>303</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2023,13 +2024,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="16" t="s">
+        <v>304</v>
+      </c>
+      <c r="C2" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="D2" s="15" t="s">
         <v>306</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2037,13 +2038,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C3" s="18">
         <v>46135</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2051,13 +2052,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C4" s="18">
         <v>46147</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2065,13 +2066,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C5" s="19">
         <v>2.7083333333333331E-2</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2079,13 +2080,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="C6" s="19" t="s">
         <v>314</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="D6" s="15" t="s">
         <v>315</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="38.4" customHeight="1">
@@ -2093,10 +2094,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="16" t="s">
+        <v>316</v>
+      </c>
+      <c r="D7" s="20" t="s">
         <v>317</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="38.4" customHeight="1">
@@ -2104,13 +2105,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="D8" s="20" t="s">
         <v>320</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>321</v>
       </c>
     </row>
   </sheetData>
@@ -2405,7 +2406,7 @@
         <v>33</v>
       </c>
       <c r="J8" s="46" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>34</v>
@@ -2440,7 +2441,7 @@
         <v>35</v>
       </c>
       <c r="J9" s="46" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>36</v>
@@ -2475,7 +2476,7 @@
         <v>37</v>
       </c>
       <c r="J10" s="46" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K10" s="8" t="s">
         <v>38</v>
@@ -2510,7 +2511,7 @@
         <v>39</v>
       </c>
       <c r="J11" s="46" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="K11" s="8" t="s">
         <v>40</v>
@@ -2580,7 +2581,7 @@
         <v>44</v>
       </c>
       <c r="J13" s="46" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>45</v>
@@ -3717,10 +3718,10 @@
         <v>128</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J46" s="46" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="K46" s="8" t="s">
         <v>141</v>
@@ -3752,10 +3753,10 @@
         <v>128</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J47" s="46" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K47" s="8" t="s">
         <v>142</v>
@@ -3790,7 +3791,7 @@
         <v>143</v>
       </c>
       <c r="J48" s="46" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K48" s="8" t="s">
         <v>144</v>
@@ -4273,10 +4274,10 @@
         <v>169</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J63" s="46" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K63" s="8" t="s">
         <v>172</v>
@@ -5497,7 +5498,7 @@
         <v>259</v>
       </c>
       <c r="J99" s="46" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="K99" s="8" t="s">
         <v>261</v>
@@ -5602,10 +5603,10 @@
         <v>270</v>
       </c>
       <c r="J102" s="46" t="s">
+        <v>333</v>
+      </c>
+      <c r="K102" s="8" t="s">
         <v>271</v>
-      </c>
-      <c r="K102" s="8" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="103" spans="1:11">
@@ -5631,16 +5632,16 @@
         <v>268</v>
       </c>
       <c r="H103" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="I103" s="10" t="s">
         <v>273</v>
       </c>
-      <c r="I103" s="10" t="s">
+      <c r="J103" s="46" t="s">
         <v>274</v>
       </c>
-      <c r="J103" s="46" t="s">
+      <c r="K103" s="8" t="s">
         <v>275</v>
-      </c>
-      <c r="K103" s="8" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="104" spans="1:11">
@@ -5660,19 +5661,19 @@
         <v>0</v>
       </c>
       <c r="F104" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="G104" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="G104" s="1" t="s">
+      <c r="H104" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H104" s="6" t="s">
+      <c r="I104" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="I104" s="10" t="s">
+      <c r="J104" s="46" t="s">
         <v>280</v>
-      </c>
-      <c r="J104" s="46" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="105" spans="1:11">
@@ -5692,19 +5693,19 @@
         <v>0</v>
       </c>
       <c r="F105" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="G105" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="G105" s="1" t="s">
+      <c r="H105" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H105" s="6" t="s">
-        <v>279</v>
-      </c>
       <c r="I105" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="J105" s="46" t="s">
         <v>282</v>
-      </c>
-      <c r="J105" s="46" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="106" spans="1:11">
@@ -5724,19 +5725,19 @@
         <v>0</v>
       </c>
       <c r="F106" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="G106" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="G106" s="1" t="s">
+      <c r="H106" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H106" s="6" t="s">
-        <v>279</v>
-      </c>
       <c r="I106" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="J106" s="46" t="s">
         <v>284</v>
-      </c>
-      <c r="J106" s="46" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="107" spans="1:11">
@@ -5756,19 +5757,19 @@
         <v>0</v>
       </c>
       <c r="F107" s="26" t="s">
+        <v>276</v>
+      </c>
+      <c r="G107" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="G107" s="1" t="s">
+      <c r="H107" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="H107" s="6" t="s">
-        <v>279</v>
-      </c>
       <c r="I107" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="J107" s="46" t="s">
         <v>286</v>
-      </c>
-      <c r="J107" s="46" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="108" spans="1:11">
@@ -5788,19 +5789,19 @@
         <v>0</v>
       </c>
       <c r="F108" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G108" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="H108" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="I108" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="H108" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="I108" s="10" t="s">
+      <c r="J108" s="46" t="s">
         <v>289</v>
-      </c>
-      <c r="J108" s="46" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="109" spans="1:11">
@@ -5820,19 +5821,19 @@
         <v>0</v>
       </c>
       <c r="F109" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G109" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I109" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="J109" s="46" t="s">
         <v>291</v>
-      </c>
-      <c r="J109" s="46" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -5852,19 +5853,19 @@
         <v>0</v>
       </c>
       <c r="F110" s="26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G110" s="1" t="s">
         <v>192</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I110" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="J110" s="46" t="s">
         <v>293</v>
-      </c>
-      <c r="J110" s="46" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="111" spans="1:11">
@@ -5884,19 +5885,19 @@
         <v>0</v>
       </c>
       <c r="F111" s="26" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G111" s="1" t="s">
         <v>123</v>
       </c>
       <c r="H111" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="I111" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="I111" s="10" t="s">
+      <c r="J111" s="46" t="s">
         <v>297</v>
-      </c>
-      <c r="J111" s="46" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="112" spans="1:11" s="45" customFormat="1" ht="19.8" customHeight="1" thickBot="1">
@@ -5916,19 +5917,19 @@
         <v>0</v>
       </c>
       <c r="F112" s="41" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G112" s="39" t="s">
         <v>123</v>
       </c>
       <c r="H112" s="40" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I112" s="42" t="s">
+        <v>298</v>
+      </c>
+      <c r="J112" s="43" t="s">
         <v>299</v>
-      </c>
-      <c r="J112" s="43" t="s">
-        <v>300</v>
       </c>
       <c r="K112" s="44"/>
     </row>

</xml_diff>